<commit_message>
Fix AnchorTP fixed-path scheduling and paused migration semantics
</commit_message>
<xml_diff>
--- a/documents/WeaveTP_实验与论文汇总.xlsx
+++ b/documents/WeaveTP_实验与论文汇总.xlsx
@@ -622,7 +622,7 @@
         <x:v>三篇对比论文</x:v>
       </x:c>
       <x:c r="B7" s="12" t="str">
-        <x:v>Flying Serving、AnchorTP、Llumnix；现有结果为同一原型的机制代理，不是官方完整性能复现。</x:v>
+        <x:v>AnchorTP 历史结果为旧代理（含 WeaveTP residual 与改道）；新实现尚无 GPU 结果，新旧不能混合比较。Flying/Llumnix 仍为机制代理。</x:v>
       </x:c>
       <x:c r="C7" s="12" t="str">
         <x:v>历史机制对照 / 各 baseline README</x:v>
@@ -2261,7 +2261,7 @@
     </x:row>
     <x:row r="20" ht="53" customHeight="1">
       <x:c r="A20" s="13" t="str">
-        <x:v>AnchorTP-proxy</x:v>
+        <x:v>AnchorTP 旧代理</x:v>
       </x:c>
       <x:c r="B20" s="13" t="str">
         <x:v>Migration base wall</x:v>
@@ -2281,12 +2281,13 @@
         <x:v>0.3452372591887691</x:v>
       </x:c>
       <x:c r="G20" s="13" t="str">
-        <x:v>全状态策略代理；不是故障恢复原系统</x:v>
+        <x:v>旧代理（含 WeaveTP residual 与改道）
+仅对应历史五轮；不与新实现混合统计</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="53" customHeight="1">
       <x:c r="A21" s="12" t="str">
-        <x:v>AnchorTP-proxy</x:v>
+        <x:v>AnchorTP 旧代理</x:v>
       </x:c>
       <x:c r="B21" s="12" t="str">
         <x:v>Transport</x:v>
@@ -2306,12 +2307,13 @@
         <x:v>0.16154916791352308</x:v>
       </x:c>
       <x:c r="G21" s="12" t="str">
-        <x:v>全状态策略代理；不是故障恢复原系统</x:v>
+        <x:v>旧代理（含 WeaveTP residual 与改道）
+仅对应历史五轮；不与新实现混合统计</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="53" customHeight="1">
       <x:c r="A22" s="13" t="str">
-        <x:v>AnchorTP-proxy</x:v>
+        <x:v>AnchorTP 旧代理</x:v>
       </x:c>
       <x:c r="B22" s="13" t="str">
         <x:v>Benchmark switch wall</x:v>
@@ -2331,12 +2333,13 @@
         <x:v>0.3510439126223612</x:v>
       </x:c>
       <x:c r="G22" s="13" t="str">
-        <x:v>全状态策略代理；不是故障恢复原系统</x:v>
+        <x:v>旧代理（含 WeaveTP residual 与改道）
+仅对应历史五轮；不与新实现混合统计</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="53" customHeight="1">
       <x:c r="A23" s="12" t="str">
-        <x:v>AnchorTP-proxy</x:v>
+        <x:v>AnchorTP 旧代理</x:v>
       </x:c>
       <x:c r="B23" s="12" t="str">
         <x:v>Foreground TPOT mean</x:v>
@@ -2356,12 +2359,13 @@
         <x:v>1.9275986297601602</x:v>
       </x:c>
       <x:c r="G23" s="12" t="str">
-        <x:v>全状态策略代理；不是故障恢复原系统</x:v>
+        <x:v>旧代理（含 WeaveTP residual 与改道）
+仅对应历史五轮；不与新实现混合统计</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="53" customHeight="1">
       <x:c r="A24" s="13" t="str">
-        <x:v>AnchorTP-proxy</x:v>
+        <x:v>AnchorTP 旧代理</x:v>
       </x:c>
       <x:c r="B24" s="13" t="str">
         <x:v>Foreground TPOT p95 摘要</x:v>
@@ -2381,7 +2385,8 @@
         <x:v>9.918993143172845</x:v>
       </x:c>
       <x:c r="G24" s="13" t="str">
-        <x:v>全状态策略代理；不是故障恢复原系统</x:v>
+        <x:v>旧代理（含 WeaveTP residual 与改道）
+仅对应历史五轮；不与新实现混合统计</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="53" customHeight="1">
@@ -2741,7 +2746,7 @@
         <x:v>三篇机制代理之一；故障恢复不是计划切换</x:v>
       </x:c>
       <x:c r="G9" s="12" t="str">
-        <x:v>机制代理有 GPU 结果</x:v>
+        <x:v>旧代理有 GPU 结果；新实现待 GPU 验收</x:v>
       </x:c>
       <x:c r="H9" s="12" t="str">
         <x:v>本次查核论文主页面</x:v>
@@ -3561,22 +3566,22 @@
         <x:v>AnchorTP</x:v>
       </x:c>
       <x:c r="B10" s="13" t="str">
-        <x:v>机制代理</x:v>
+        <x:v>旧代理 + 新实现</x:v>
       </x:c>
       <x:c r="C10" s="13" t="str">
-        <x:v>参数/KV 路径与 residual/aware 配置</x:v>
+        <x:v>旧代理（含 WeaveTP residual 与改道）</x:v>
       </x:c>
       <x:c r="D10" s="13" t="str">
-        <x:v>历史五轮，真实 GPU benchmark</x:v>
+        <x:v>历史五轮仅为旧代理 GPU 结果</x:v>
       </x:c>
       <x:c r="E10" s="13" t="str">
         <x:v>同历史平台</x:v>
       </x:c>
       <x:c r="F10" s="13" t="str">
-        <x:v>有代理结果；非官方复现</x:v>
+        <x:v>新实现代码/CPU 验收；GPU 待验收</x:v>
       </x:c>
       <x:c r="G10" s="13" t="str">
-        <x:v>没有复现完整故障恢复及非等宽弹性协议</x:v>
+        <x:v>新实现：固定源三类路径、整体预分配、停服；故障检测/CMM 缺口生成/非等宽 TP 未实现</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="85" customHeight="1">
@@ -4762,7 +4767,7 @@
         <x:v>历史五轮机制代理</x:v>
       </x:c>
       <x:c r="B35" s="12" t="str">
-        <x:v>AnchorTP-proxy</x:v>
+        <x:v>AnchorTP 旧代理</x:v>
       </x:c>
       <x:c r="C35" s="19" t="n">
         <x:v>1</x:v>
@@ -4890,7 +4895,7 @@
         <x:v>历史五轮机制代理</x:v>
       </x:c>
       <x:c r="B39" s="12" t="str">
-        <x:v>AnchorTP-proxy</x:v>
+        <x:v>AnchorTP 旧代理</x:v>
       </x:c>
       <x:c r="C39" s="19" t="n">
         <x:v>2</x:v>
@@ -4922,7 +4927,7 @@
         <x:v>历史五轮机制代理</x:v>
       </x:c>
       <x:c r="B40" s="13" t="str">
-        <x:v>AnchorTP-proxy</x:v>
+        <x:v>AnchorTP 旧代理</x:v>
       </x:c>
       <x:c r="C40" s="20" t="n">
         <x:v>3</x:v>
@@ -5146,7 +5151,7 @@
         <x:v>历史五轮机制代理</x:v>
       </x:c>
       <x:c r="B47" s="12" t="str">
-        <x:v>AnchorTP-proxy</x:v>
+        <x:v>AnchorTP 旧代理</x:v>
       </x:c>
       <x:c r="C47" s="19" t="n">
         <x:v>4</x:v>
@@ -5274,7 +5279,7 @@
         <x:v>历史五轮机制代理</x:v>
       </x:c>
       <x:c r="B51" s="12" t="str">
-        <x:v>AnchorTP-proxy</x:v>
+        <x:v>AnchorTP 旧代理</x:v>
       </x:c>
       <x:c r="C51" s="19" t="n">
         <x:v>5</x:v>

</xml_diff>